<commit_message>
fix: enforce real cell protection on all BRASUS sheets (v2.1)
Previously cells used only visual grey fill to suggest read-only status
but had no actual worksheet protection — all cells remained editable.

Changes:
- Activate ws.protection.sheet = True on every worksheet
- All cells explicitly set Protection(locked=True) by default
- Only truly editable cells (fond jaune INPUT_YLW) set to locked=False:
  • Missions du jour: colonnes STATUT + COMMENTAIRE (col F+G, rows 5-12)
  • Exécution journalière: Sections A, B (résultat+statut), C, D
  • Cockpit DG plan d'actions: colonne STATUT uniquement (col F)
- Sheets 3/4/5 and all Cockpit sheets: 100% read-only (all locked=True)
- Performances sheet: reco cells changed from INPUT_YLW to LOCKED_BG
  (they are generated by BRASUS, not user-editable)
- Admin unlock password: BRASUS_ADMIN_2026 (to change per client)

https://claude.ai/code/session_01BSsMiXSsDbXvN6rY3KW34P
</commit_message>
<xml_diff>
--- a/brasus/skills/google-workspace/sheets/BRASUS_COCKPIT_DG.xlsx
+++ b/brasus/skills/google-workspace/sheets/BRASUS_COCKPIT_DG.xlsx
@@ -492,8 +492,9 @@
     <xf numFmtId="0" fontId="13" fillId="11" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="15" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -1167,11 +1168,12 @@
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
-          <t>🔒 Données consolidées par BRASUS — Lecture seule</t>
+          <t>🔒 Données consolidées par BRASUS — Lecture seule intégrale</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCC2"/>
   <mergeCells count="5">
     <mergeCell ref="E2:F2"/>
     <mergeCell ref="A1:F1"/>
@@ -1521,6 +1523,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCC2"/>
   <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B16:F16"/>
@@ -1874,6 +1877,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCC2"/>
   <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B16:F16"/>
@@ -2227,6 +2231,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCC2"/>
   <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B16:F16"/>
@@ -2580,6 +2585,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCC2"/>
   <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B16:F16"/>
@@ -2933,6 +2939,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCC2"/>
   <mergeCells count="9">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="B16:F16"/>
@@ -3102,6 +3109,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCC2"/>
   <mergeCells count="19">
     <mergeCell ref="A15:B15"/>
     <mergeCell ref="A11:B11"/>
@@ -3387,11 +3395,12 @@
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="56" t="inlineStr">
         <is>
-          <t>Colonne STATUT modifiable par le DG — Toutes les autres colonnes en lecture seule</t>
+          <t>Colonne STATUT (fond jaune) modifiable par le DG — Toutes les autres colonnes en lecture seule</t>
         </is>
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1" password="CCC2"/>
   <mergeCells count="3">
     <mergeCell ref="A2:F2"/>
     <mergeCell ref="A11:F11"/>

</xml_diff>